<commit_message>
merge data in idc final version
</commit_message>
<xml_diff>
--- a/codebooks/c_educacion/2023_adopcion_digital.xlsx
+++ b/codebooks/c_educacion/2023_adopcion_digital.xlsx
@@ -277,6 +277,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -550,7 +554,7 @@
     <col min="5" max="5" width="43.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="173" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:6" ht="69.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -570,7 +574,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="173" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:6" ht="69.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -590,7 +594,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="173" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:6" ht="69.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -610,7 +614,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="173" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:6" ht="69.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
@@ -630,7 +634,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="173" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:6" ht="69.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -650,7 +654,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="173" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:6" ht="69.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -670,7 +674,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="173" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:6" ht="69.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="1" t="s">
         <v>0</v>
       </c>
@@ -690,7 +694,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="173" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:6" ht="69.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="1" t="s">
         <v>18</v>
       </c>
@@ -710,7 +714,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="173" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:6" ht="69.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="1" t="s">
         <v>18</v>
       </c>
@@ -730,7 +734,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="173" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:6" ht="69.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
@@ -750,7 +754,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="173" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:6" ht="69.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="1" t="s">
         <v>18</v>
       </c>
@@ -770,7 +774,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="173" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:6" ht="69.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="1" t="s">
         <v>18</v>
       </c>
@@ -790,7 +794,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="173" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:6" ht="69.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="1" t="s">
         <v>18</v>
       </c>
@@ -810,7 +814,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="173" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:6" ht="69.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="1" t="s">
         <v>32</v>
       </c>
@@ -830,7 +834,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="173" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:6" ht="69.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="1" t="s">
         <v>32</v>
       </c>
@@ -850,7 +854,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="173" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:6" ht="69.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A16" s="1" t="s">
         <v>32</v>
       </c>
@@ -870,7 +874,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="173" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:6" ht="69.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A17" s="1" t="s">
         <v>32</v>
       </c>
@@ -890,7 +894,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="173" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:6" ht="69.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A18" s="1" t="s">
         <v>32</v>
       </c>
@@ -910,7 +914,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="173" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:6" ht="69.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A19" s="1" t="s">
         <v>32</v>
       </c>

</xml_diff>